<commit_message>
features: delete and create sino vietnamese
</commit_message>
<xml_diff>
--- a/sources/sino/main_sino_vietnamese.xlsx
+++ b/sources/sino/main_sino_vietnamese.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ki_8\JPD326\Code\Japan-Go\sources\sino\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ki_9\SEP490\Japan-Go\sources\sino\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3540616C-97AD-44C2-86B1-D2F049123F2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0059E7C-F2C1-4C1A-96AC-01F3350BBACD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="N5 - N2" sheetId="1" r:id="rId1"/>
@@ -17396,7 +17396,7 @@
         <v>881</v>
       </c>
       <c r="C479" s="1" t="s">
-        <v>882</v>
+        <v>404</v>
       </c>
     </row>
     <row r="480" spans="1:3" s="1" customFormat="1" ht="26.15" x14ac:dyDescent="0.4">

</xml_diff>